<commit_message>
Updated on 10-27-2023 at 17:40
</commit_message>
<xml_diff>
--- a/data/dados_full_brasil.xlsx
+++ b/data/dados_full_brasil.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Gustavo\AppData\Local\Temp\scp33883\home\gustavo\Documents\lovo_code\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\home\gustavo\LOVO\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B039BA4-3784-46AC-81C0-D4F2A245735D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EB1A9DF-3FB0-4DCA-9486-1DA9DC677BB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4210,7 +4210,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
@@ -4219,6 +4219,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -30900,2122 +30901,2122 @@
       </c>
     </row>
     <row r="517" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A517" t="s">
-        <v>17</v>
-      </c>
-      <c r="B517" t="s">
-        <v>18</v>
-      </c>
-      <c r="C517" t="s">
-        <v>19</v>
-      </c>
-      <c r="D517" t="s">
+      <c r="A517" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B517" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C517" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D517" s="4" t="s">
         <v>481</v>
       </c>
-      <c r="E517">
+      <c r="E517" s="4">
         <v>16515120</v>
       </c>
-      <c r="F517">
+      <c r="F517" s="4">
         <v>43520</v>
       </c>
-      <c r="G517">
+      <c r="G517" s="4">
         <v>61694.571000000004</v>
       </c>
-      <c r="H517">
+      <c r="H517" s="4">
         <v>461931</v>
       </c>
-      <c r="I517">
+      <c r="I517" s="4">
         <v>874</v>
       </c>
-      <c r="J517">
+      <c r="J517" s="4">
         <v>1837.5709999999999</v>
       </c>
-      <c r="K517">
+      <c r="K517" s="4">
         <v>76702.667000000001</v>
       </c>
-      <c r="L517">
+      <c r="L517" s="4">
         <v>202.124</v>
       </c>
-      <c r="M517">
+      <c r="M517" s="4">
         <v>286.53399999999999</v>
       </c>
-      <c r="N517">
+      <c r="N517" s="4">
         <v>2145.3879999999999</v>
       </c>
-      <c r="O517">
+      <c r="O517" s="4">
         <v>4.0590000000000002</v>
       </c>
-      <c r="P517">
+      <c r="P517" s="4">
         <v>8.5340000000000007</v>
       </c>
-      <c r="Q517">
+      <c r="Q517" s="4">
         <v>1.01</v>
       </c>
     </row>
     <row r="518" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A518" t="s">
-        <v>17</v>
-      </c>
-      <c r="B518" t="s">
-        <v>18</v>
-      </c>
-      <c r="C518" t="s">
-        <v>19</v>
-      </c>
-      <c r="D518" t="s">
+      <c r="A518" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B518" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C518" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D518" s="4" t="s">
         <v>482</v>
       </c>
-      <c r="E518">
+      <c r="E518" s="4">
         <v>16545554</v>
       </c>
-      <c r="F518">
+      <c r="F518" s="4">
         <v>30434</v>
       </c>
-      <c r="G518">
+      <c r="G518" s="4">
         <v>60685.428999999996</v>
       </c>
-      <c r="H518">
+      <c r="H518" s="4">
         <v>462791</v>
       </c>
-      <c r="I518">
+      <c r="I518" s="4">
         <v>860</v>
       </c>
-      <c r="J518">
+      <c r="J518" s="4">
         <v>1847.5709999999999</v>
       </c>
-      <c r="K518">
+      <c r="K518" s="4">
         <v>76844.013999999996</v>
       </c>
-      <c r="L518">
+      <c r="L518" s="4">
         <v>141.34700000000001</v>
       </c>
-      <c r="M518">
+      <c r="M518" s="4">
         <v>281.84699999999998</v>
       </c>
-      <c r="N518">
+      <c r="N518" s="4">
         <v>2149.3820000000001</v>
       </c>
-      <c r="O518">
+      <c r="O518" s="4">
         <v>3.9940000000000002</v>
       </c>
-      <c r="P518">
+      <c r="P518" s="4">
         <v>8.5809999999999995</v>
       </c>
-      <c r="Q518">
+      <c r="Q518" s="4">
         <v>1.01</v>
       </c>
     </row>
     <row r="519" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A519" t="s">
-        <v>17</v>
-      </c>
-      <c r="B519" t="s">
-        <v>18</v>
-      </c>
-      <c r="C519" t="s">
-        <v>19</v>
-      </c>
-      <c r="D519" t="s">
+      <c r="A519" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B519" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C519" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D519" s="4" t="s">
         <v>483</v>
       </c>
-      <c r="E519">
+      <c r="E519" s="4">
         <v>16624480</v>
       </c>
-      <c r="F519">
+      <c r="F519" s="4">
         <v>78926</v>
       </c>
-      <c r="G519">
+      <c r="G519" s="4">
         <v>61467.286</v>
       </c>
-      <c r="H519">
+      <c r="H519" s="4">
         <v>465199</v>
       </c>
-      <c r="I519">
+      <c r="I519" s="4">
         <v>2408</v>
       </c>
-      <c r="J519">
+      <c r="J519" s="4">
         <v>1881.143</v>
       </c>
-      <c r="K519">
+      <c r="K519" s="4">
         <v>77210.577999999994</v>
       </c>
-      <c r="L519">
+      <c r="L519" s="4">
         <v>366.56299999999999</v>
       </c>
-      <c r="M519">
+      <c r="M519" s="4">
         <v>285.47800000000001</v>
       </c>
-      <c r="N519">
+      <c r="N519" s="4">
         <v>2160.5659999999998</v>
       </c>
-      <c r="O519">
+      <c r="O519" s="4">
         <v>11.183999999999999</v>
       </c>
-      <c r="P519">
+      <c r="P519" s="4">
         <v>8.7370000000000001</v>
       </c>
-      <c r="Q519">
+      <c r="Q519" s="4">
         <v>1.01</v>
       </c>
     </row>
     <row r="520" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A520" t="s">
-        <v>17</v>
-      </c>
-      <c r="B520" t="s">
-        <v>18</v>
-      </c>
-      <c r="C520" t="s">
-        <v>19</v>
-      </c>
-      <c r="D520" t="s">
+      <c r="A520" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B520" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C520" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D520" s="4" t="s">
         <v>484</v>
       </c>
-      <c r="E520">
+      <c r="E520" s="4">
         <v>16720081</v>
       </c>
-      <c r="F520">
+      <c r="F520" s="4">
         <v>95601</v>
       </c>
-      <c r="G520">
+      <c r="G520" s="4">
         <v>63626.571000000004</v>
       </c>
-      <c r="H520">
+      <c r="H520" s="4">
         <v>467706</v>
       </c>
-      <c r="I520">
+      <c r="I520" s="4">
         <v>2507</v>
       </c>
-      <c r="J520">
+      <c r="J520" s="4">
         <v>1896.7139999999999</v>
       </c>
-      <c r="K520">
+      <c r="K520" s="4">
         <v>77654.585999999996</v>
       </c>
-      <c r="L520">
+      <c r="L520" s="4">
         <v>444.00799999999998</v>
       </c>
-      <c r="M520">
+      <c r="M520" s="4">
         <v>295.50700000000001</v>
       </c>
-      <c r="N520">
+      <c r="N520" s="4">
         <v>2172.2089999999998</v>
       </c>
-      <c r="O520">
+      <c r="O520" s="4">
         <v>11.643000000000001</v>
       </c>
-      <c r="P520">
+      <c r="P520" s="4">
         <v>8.8089999999999993</v>
       </c>
-      <c r="Q520">
+      <c r="Q520" s="4">
         <v>1</v>
       </c>
     </row>
     <row r="521" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A521" t="s">
-        <v>17</v>
-      </c>
-      <c r="B521" t="s">
-        <v>18</v>
-      </c>
-      <c r="C521" t="s">
-        <v>19</v>
-      </c>
-      <c r="D521" t="s">
+      <c r="A521" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B521" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C521" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D521" s="4" t="s">
         <v>485</v>
       </c>
-      <c r="E521">
+      <c r="E521" s="4">
         <v>16803472</v>
       </c>
-      <c r="F521">
+      <c r="F521" s="4">
         <v>83391</v>
       </c>
-      <c r="G521">
+      <c r="G521" s="4">
         <v>65901.429000000004</v>
       </c>
-      <c r="H521">
+      <c r="H521" s="4">
         <v>469388</v>
       </c>
-      <c r="I521">
+      <c r="I521" s="4">
         <v>1682</v>
       </c>
-      <c r="J521">
+      <c r="J521" s="4">
         <v>1816.2860000000001</v>
       </c>
-      <c r="K521">
+      <c r="K521" s="4">
         <v>78041.885999999999</v>
       </c>
-      <c r="L521">
+      <c r="L521" s="4">
         <v>387.3</v>
       </c>
-      <c r="M521">
+      <c r="M521" s="4">
         <v>306.072</v>
       </c>
-      <c r="N521">
+      <c r="N521" s="4">
         <v>2180.0210000000002</v>
       </c>
-      <c r="O521">
+      <c r="O521" s="4">
         <v>7.8120000000000003</v>
       </c>
-      <c r="P521">
+      <c r="P521" s="4">
         <v>8.4359999999999999</v>
       </c>
-      <c r="Q521">
+      <c r="Q521" s="4">
         <v>1.01</v>
       </c>
     </row>
     <row r="522" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A522" t="s">
-        <v>17</v>
-      </c>
-      <c r="B522" t="s">
-        <v>18</v>
-      </c>
-      <c r="C522" t="s">
-        <v>19</v>
-      </c>
-      <c r="D522" t="s">
+      <c r="A522" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B522" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C522" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D522" s="4" t="s">
         <v>486</v>
       </c>
-      <c r="E522">
+      <c r="E522" s="4">
         <v>16841408</v>
       </c>
-      <c r="F522">
+      <c r="F522" s="4">
         <v>37936</v>
       </c>
-      <c r="G522">
+      <c r="G522" s="4">
         <v>64211.142999999996</v>
       </c>
-      <c r="H522">
+      <c r="H522" s="4">
         <v>470842</v>
       </c>
-      <c r="I522">
+      <c r="I522" s="4">
         <v>1454</v>
       </c>
-      <c r="J522">
+      <c r="J522" s="4">
         <v>1685.2860000000001</v>
       </c>
-      <c r="K522">
+      <c r="K522" s="4">
         <v>78218.076000000001</v>
       </c>
-      <c r="L522">
+      <c r="L522" s="4">
         <v>176.19</v>
       </c>
-      <c r="M522">
+      <c r="M522" s="4">
         <v>298.22199999999998</v>
       </c>
-      <c r="N522">
+      <c r="N522" s="4">
         <v>2186.7739999999999</v>
       </c>
-      <c r="O522">
+      <c r="O522" s="4">
         <v>6.7530000000000001</v>
       </c>
-      <c r="P522">
+      <c r="P522" s="4">
         <v>7.827</v>
       </c>
-      <c r="Q522">
+      <c r="Q522" s="4">
         <v>1.01</v>
       </c>
     </row>
     <row r="523" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A523" t="s">
-        <v>17</v>
-      </c>
-      <c r="B523" t="s">
-        <v>18</v>
-      </c>
-      <c r="C523" t="s">
-        <v>19</v>
-      </c>
-      <c r="D523" t="s">
+      <c r="A523" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B523" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C523" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D523" s="4" t="s">
         <v>487</v>
       </c>
-      <c r="E523">
+      <c r="E523" s="4">
         <v>16907425</v>
       </c>
-      <c r="F523">
+      <c r="F523" s="4">
         <v>66017</v>
       </c>
-      <c r="G523">
+      <c r="G523" s="4">
         <v>62260.714</v>
       </c>
-      <c r="H523">
+      <c r="H523" s="4">
         <v>472531</v>
       </c>
-      <c r="I523">
+      <c r="I523" s="4">
         <v>1689</v>
       </c>
-      <c r="J523">
+      <c r="J523" s="4">
         <v>1639.143</v>
       </c>
-      <c r="K523">
+      <c r="K523" s="4">
         <v>78524.684999999998</v>
       </c>
-      <c r="L523">
+      <c r="L523" s="4">
         <v>306.60899999999998</v>
       </c>
-      <c r="M523">
+      <c r="M523" s="4">
         <v>289.16300000000001</v>
       </c>
-      <c r="N523">
+      <c r="N523" s="4">
         <v>2194.6190000000001</v>
       </c>
-      <c r="O523">
+      <c r="O523" s="4">
         <v>7.8440000000000003</v>
       </c>
-      <c r="P523">
+      <c r="P523" s="4">
         <v>7.6130000000000004</v>
       </c>
-      <c r="Q523">
+      <c r="Q523" s="4">
         <v>1.01</v>
       </c>
     </row>
     <row r="524" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A524" t="s">
-        <v>17</v>
-      </c>
-      <c r="B524" t="s">
-        <v>18</v>
-      </c>
-      <c r="C524" t="s">
-        <v>19</v>
-      </c>
-      <c r="D524" t="s">
+      <c r="A524" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B524" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C524" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D524" s="4" t="s">
         <v>488</v>
       </c>
-      <c r="E524">
+      <c r="E524" s="4">
         <v>16947062</v>
       </c>
-      <c r="F524">
+      <c r="F524" s="4">
         <v>39637</v>
       </c>
-      <c r="G524">
+      <c r="G524" s="4">
         <v>61706</v>
       </c>
-      <c r="H524">
+      <c r="H524" s="4">
         <v>473404</v>
       </c>
-      <c r="I524">
+      <c r="I524" s="4">
         <v>873</v>
       </c>
-      <c r="J524">
+      <c r="J524" s="4">
         <v>1639</v>
       </c>
-      <c r="K524">
+      <c r="K524" s="4">
         <v>78708.774000000005</v>
       </c>
-      <c r="L524">
+      <c r="L524" s="4">
         <v>184.09</v>
       </c>
-      <c r="M524">
+      <c r="M524" s="4">
         <v>286.58699999999999</v>
       </c>
-      <c r="N524">
+      <c r="N524" s="4">
         <v>2198.6729999999998</v>
       </c>
-      <c r="O524">
+      <c r="O524" s="4">
         <v>4.0549999999999997</v>
       </c>
-      <c r="P524">
+      <c r="P524" s="4">
         <v>7.6120000000000001</v>
       </c>
-      <c r="Q524">
+      <c r="Q524" s="4">
         <v>1.01</v>
       </c>
     </row>
     <row r="525" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A525" t="s">
-        <v>17</v>
-      </c>
-      <c r="B525" t="s">
-        <v>18</v>
-      </c>
-      <c r="C525" t="s">
-        <v>19</v>
-      </c>
-      <c r="D525" t="s">
+      <c r="A525" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B525" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C525" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D525" s="4" t="s">
         <v>489</v>
       </c>
-      <c r="E525">
+      <c r="E525" s="4">
         <v>16984218</v>
       </c>
-      <c r="F525">
+      <c r="F525" s="4">
         <v>37156</v>
       </c>
-      <c r="G525">
+      <c r="G525" s="4">
         <v>62666.286</v>
       </c>
-      <c r="H525">
+      <c r="H525" s="4">
         <v>474414</v>
       </c>
-      <c r="I525">
+      <c r="I525" s="4">
         <v>1010</v>
       </c>
-      <c r="J525">
+      <c r="J525" s="4">
         <v>1660.4290000000001</v>
       </c>
-      <c r="K525">
+      <c r="K525" s="4">
         <v>78881.341</v>
       </c>
-      <c r="L525">
+      <c r="L525" s="4">
         <v>172.56700000000001</v>
       </c>
-      <c r="M525">
+      <c r="M525" s="4">
         <v>291.04700000000003</v>
       </c>
-      <c r="N525">
+      <c r="N525" s="4">
         <v>2203.364</v>
       </c>
-      <c r="O525">
+      <c r="O525" s="4">
         <v>4.6909999999999998</v>
       </c>
-      <c r="P525">
+      <c r="P525" s="4">
         <v>7.7119999999999997</v>
       </c>
-      <c r="Q525">
+      <c r="Q525" s="4">
         <v>1.01</v>
       </c>
     </row>
     <row r="526" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A526" t="s">
-        <v>17</v>
-      </c>
-      <c r="B526" t="s">
-        <v>18</v>
-      </c>
-      <c r="C526" t="s">
-        <v>19</v>
-      </c>
-      <c r="D526" t="s">
+      <c r="A526" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B526" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C526" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D526" s="4" t="s">
         <v>490</v>
       </c>
-      <c r="E526">
+      <c r="E526" s="4">
         <v>17037129</v>
       </c>
-      <c r="F526">
+      <c r="F526" s="4">
         <v>52911</v>
       </c>
-      <c r="G526">
+      <c r="G526" s="4">
         <v>58949.857000000004</v>
       </c>
-      <c r="H526">
+      <c r="H526" s="4">
         <v>476792</v>
       </c>
-      <c r="I526">
+      <c r="I526" s="4">
         <v>2378</v>
       </c>
-      <c r="J526">
+      <c r="J526" s="4">
         <v>1656.143</v>
       </c>
-      <c r="K526">
+      <c r="K526" s="4">
         <v>79127.081000000006</v>
       </c>
-      <c r="L526">
+      <c r="L526" s="4">
         <v>245.739</v>
       </c>
-      <c r="M526">
+      <c r="M526" s="4">
         <v>273.786</v>
       </c>
-      <c r="N526">
+      <c r="N526" s="4">
         <v>2214.4079999999999</v>
       </c>
-      <c r="O526">
+      <c r="O526" s="4">
         <v>11.044</v>
       </c>
-      <c r="P526">
+      <c r="P526" s="4">
         <v>7.6920000000000002</v>
       </c>
-      <c r="Q526">
+      <c r="Q526" s="4">
         <v>1.02</v>
       </c>
     </row>
     <row r="527" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A527" t="s">
-        <v>17</v>
-      </c>
-      <c r="B527" t="s">
-        <v>18</v>
-      </c>
-      <c r="C527" t="s">
-        <v>19</v>
-      </c>
-      <c r="D527" t="s">
+      <c r="A527" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B527" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C527" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D527" s="4" t="s">
         <v>491</v>
       </c>
-      <c r="E527">
+      <c r="E527" s="4">
         <v>17122877</v>
       </c>
-      <c r="F527">
+      <c r="F527" s="4">
         <v>85748</v>
       </c>
-      <c r="G527">
+      <c r="G527" s="4">
         <v>57542.286</v>
       </c>
-      <c r="H527">
+      <c r="H527" s="4">
         <v>479515</v>
       </c>
-      <c r="I527">
+      <c r="I527" s="4">
         <v>2723</v>
       </c>
-      <c r="J527">
+      <c r="J527" s="4">
         <v>1687</v>
       </c>
-      <c r="K527">
+      <c r="K527" s="4">
         <v>79525.327999999994</v>
       </c>
-      <c r="L527">
+      <c r="L527" s="4">
         <v>398.24700000000001</v>
       </c>
-      <c r="M527">
+      <c r="M527" s="4">
         <v>267.24900000000002</v>
       </c>
-      <c r="N527">
+      <c r="N527" s="4">
         <v>2227.0549999999998</v>
       </c>
-      <c r="O527">
+      <c r="O527" s="4">
         <v>12.647</v>
       </c>
-      <c r="P527">
+      <c r="P527" s="4">
         <v>7.835</v>
       </c>
-      <c r="Q527">
+      <c r="Q527" s="4">
         <v>1.02</v>
       </c>
     </row>
     <row r="528" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A528" t="s">
-        <v>17</v>
-      </c>
-      <c r="B528" t="s">
-        <v>18</v>
-      </c>
-      <c r="C528" t="s">
-        <v>19</v>
-      </c>
-      <c r="D528" t="s">
+      <c r="A528" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B528" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C528" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D528" s="4" t="s">
         <v>492</v>
       </c>
-      <c r="E528">
+      <c r="E528" s="4">
         <v>17210969</v>
       </c>
-      <c r="F528">
+      <c r="F528" s="4">
         <v>88092</v>
       </c>
-      <c r="G528">
+      <c r="G528" s="4">
         <v>58213.857000000004</v>
       </c>
-      <c r="H528">
+      <c r="H528" s="4">
         <v>482019</v>
       </c>
-      <c r="I528">
+      <c r="I528" s="4">
         <v>2504</v>
       </c>
-      <c r="J528">
+      <c r="J528" s="4">
         <v>1804.4290000000001</v>
       </c>
-      <c r="K528">
+      <c r="K528" s="4">
         <v>79934.462</v>
       </c>
-      <c r="L528">
+      <c r="L528" s="4">
         <v>409.13400000000001</v>
       </c>
-      <c r="M528">
+      <c r="M528" s="4">
         <v>270.36799999999999</v>
       </c>
-      <c r="N528">
+      <c r="N528" s="4">
         <v>2238.6840000000002</v>
       </c>
-      <c r="O528">
+      <c r="O528" s="4">
         <v>11.63</v>
       </c>
-      <c r="P528">
+      <c r="P528" s="4">
         <v>8.3800000000000008</v>
       </c>
-      <c r="Q528">
+      <c r="Q528" s="4">
         <v>1.01</v>
       </c>
     </row>
     <row r="529" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A529" t="s">
-        <v>17</v>
-      </c>
-      <c r="B529" t="s">
-        <v>18</v>
-      </c>
-      <c r="C529" t="s">
-        <v>19</v>
-      </c>
-      <c r="D529" t="s">
+      <c r="A529" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B529" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C529" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D529" s="4" t="s">
         <v>493</v>
       </c>
-      <c r="E529">
+      <c r="E529" s="4">
         <v>17296118</v>
       </c>
-      <c r="F529">
+      <c r="F529" s="4">
         <v>85149</v>
       </c>
-      <c r="G529">
+      <c r="G529" s="4">
         <v>64958.571000000004</v>
       </c>
-      <c r="H529">
+      <c r="H529" s="4">
         <v>484235</v>
       </c>
-      <c r="I529">
+      <c r="I529" s="4">
         <v>2216</v>
       </c>
-      <c r="J529">
+      <c r="J529" s="4">
         <v>1913.2860000000001</v>
       </c>
-      <c r="K529">
+      <c r="K529" s="4">
         <v>80329.926999999996</v>
       </c>
-      <c r="L529">
+      <c r="L529" s="4">
         <v>395.46499999999997</v>
       </c>
-      <c r="M529">
+      <c r="M529" s="4">
         <v>301.69299999999998</v>
       </c>
-      <c r="N529">
+      <c r="N529" s="4">
         <v>2248.9760000000001</v>
       </c>
-      <c r="O529">
+      <c r="O529" s="4">
         <v>10.292</v>
       </c>
-      <c r="P529">
+      <c r="P529" s="4">
         <v>8.8859999999999992</v>
       </c>
-      <c r="Q529">
+      <c r="Q529" s="4">
         <v>1.01</v>
       </c>
     </row>
     <row r="530" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A530" t="s">
-        <v>17</v>
-      </c>
-      <c r="B530" t="s">
-        <v>18</v>
-      </c>
-      <c r="C530" t="s">
-        <v>19</v>
-      </c>
-      <c r="D530" t="s">
+      <c r="A530" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B530" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C530" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D530" s="4" t="s">
         <v>494</v>
       </c>
-      <c r="E530">
+      <c r="E530" s="4">
         <v>17374818</v>
       </c>
-      <c r="F530">
+      <c r="F530" s="4">
         <v>78700</v>
       </c>
-      <c r="G530">
+      <c r="G530" s="4">
         <v>66770.429000000004</v>
       </c>
-      <c r="H530">
+      <c r="H530" s="4">
         <v>486272</v>
       </c>
-      <c r="I530">
+      <c r="I530" s="4">
         <v>2037</v>
       </c>
-      <c r="J530">
+      <c r="J530" s="4">
         <v>1963</v>
       </c>
-      <c r="K530">
+      <c r="K530" s="4">
         <v>80695.44</v>
       </c>
-      <c r="L530">
+      <c r="L530" s="4">
         <v>365.51400000000001</v>
       </c>
-      <c r="M530">
+      <c r="M530" s="4">
         <v>310.108</v>
       </c>
-      <c r="N530">
+      <c r="N530" s="4">
         <v>2258.4369999999999</v>
       </c>
-      <c r="O530">
+      <c r="O530" s="4">
         <v>9.4610000000000003</v>
       </c>
-      <c r="P530">
+      <c r="P530" s="4">
         <v>9.1170000000000009</v>
       </c>
-      <c r="Q530">
+      <c r="Q530" s="4">
         <v>1.01</v>
       </c>
     </row>
     <row r="531" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A531" t="s">
-        <v>17</v>
-      </c>
-      <c r="B531" t="s">
-        <v>18</v>
-      </c>
-      <c r="C531" t="s">
-        <v>19</v>
-      </c>
-      <c r="D531" t="s">
+      <c r="A531" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B531" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C531" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D531" s="4" t="s">
         <v>495</v>
       </c>
-      <c r="E531">
+      <c r="E531" s="4">
         <v>17412766</v>
       </c>
-      <c r="F531">
+      <c r="F531" s="4">
         <v>37948</v>
       </c>
-      <c r="G531">
+      <c r="G531" s="4">
         <v>66529.142999999996</v>
       </c>
-      <c r="H531">
+      <c r="H531" s="4">
         <v>487401</v>
       </c>
-      <c r="I531">
+      <c r="I531" s="4">
         <v>1129</v>
       </c>
-      <c r="J531">
+      <c r="J531" s="4">
         <v>1999.5709999999999</v>
       </c>
-      <c r="K531">
+      <c r="K531" s="4">
         <v>80871.686000000002</v>
       </c>
-      <c r="L531">
+      <c r="L531" s="4">
         <v>176.245</v>
       </c>
-      <c r="M531">
+      <c r="M531" s="4">
         <v>308.98700000000002</v>
       </c>
-      <c r="N531">
+      <c r="N531" s="4">
         <v>2263.681</v>
       </c>
-      <c r="O531">
+      <c r="O531" s="4">
         <v>5.2439999999999998</v>
       </c>
-      <c r="P531">
+      <c r="P531" s="4">
         <v>9.2870000000000008</v>
       </c>
-      <c r="Q531">
+      <c r="Q531" s="4">
         <v>1.01</v>
       </c>
     </row>
     <row r="532" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A532" t="s">
-        <v>17</v>
-      </c>
-      <c r="B532" t="s">
-        <v>18</v>
-      </c>
-      <c r="C532" t="s">
-        <v>19</v>
-      </c>
-      <c r="D532" t="s">
+      <c r="A532" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B532" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C532" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D532" s="4" t="s">
         <v>496</v>
       </c>
-      <c r="E532">
+      <c r="E532" s="4">
         <v>17452612</v>
       </c>
-      <c r="F532">
+      <c r="F532" s="4">
         <v>39846</v>
       </c>
-      <c r="G532">
+      <c r="G532" s="4">
         <v>66913.429000000004</v>
       </c>
-      <c r="H532">
+      <c r="H532" s="4">
         <v>488228</v>
       </c>
-      <c r="I532">
+      <c r="I532" s="4">
         <v>827</v>
       </c>
-      <c r="J532">
+      <c r="J532" s="4">
         <v>1973.4290000000001</v>
       </c>
-      <c r="K532">
+      <c r="K532" s="4">
         <v>81056.745999999999</v>
       </c>
-      <c r="L532">
+      <c r="L532" s="4">
         <v>185.06</v>
       </c>
-      <c r="M532">
+      <c r="M532" s="4">
         <v>310.77199999999999</v>
       </c>
-      <c r="N532">
+      <c r="N532" s="4">
         <v>2267.5219999999999</v>
       </c>
-      <c r="O532">
+      <c r="O532" s="4">
         <v>3.8410000000000002</v>
       </c>
-      <c r="P532">
+      <c r="P532" s="4">
         <v>9.1649999999999991</v>
       </c>
-      <c r="Q532">
+      <c r="Q532" s="4">
         <v>1.01</v>
       </c>
     </row>
     <row r="533" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A533" t="s">
-        <v>17</v>
-      </c>
-      <c r="B533" t="s">
-        <v>18</v>
-      </c>
-      <c r="C533" t="s">
-        <v>19</v>
-      </c>
-      <c r="D533" t="s">
+      <c r="A533" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B533" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C533" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D533" s="4" t="s">
         <v>497</v>
       </c>
-      <c r="E533">
+      <c r="E533" s="4">
         <v>17533221</v>
       </c>
-      <c r="F533">
+      <c r="F533" s="4">
         <v>80609</v>
       </c>
-      <c r="G533">
+      <c r="G533" s="4">
         <v>70870.285999999993</v>
       </c>
-      <c r="H533">
+      <c r="H533" s="4">
         <v>490696</v>
       </c>
-      <c r="I533">
+      <c r="I533" s="4">
         <v>2468</v>
       </c>
-      <c r="J533">
+      <c r="J533" s="4">
         <v>1986.2860000000001</v>
       </c>
-      <c r="K533">
+      <c r="K533" s="4">
         <v>81431.126000000004</v>
       </c>
-      <c r="L533">
+      <c r="L533" s="4">
         <v>374.38</v>
       </c>
-      <c r="M533">
+      <c r="M533" s="4">
         <v>329.149</v>
       </c>
-      <c r="N533">
+      <c r="N533" s="4">
         <v>2278.9839999999999</v>
       </c>
-      <c r="O533">
+      <c r="O533" s="4">
         <v>11.462</v>
       </c>
-      <c r="P533">
+      <c r="P533" s="4">
         <v>9.2249999999999996</v>
       </c>
-      <c r="Q533">
+      <c r="Q533" s="4">
         <v>1</v>
       </c>
     </row>
     <row r="534" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A534" t="s">
-        <v>17</v>
-      </c>
-      <c r="B534" t="s">
-        <v>18</v>
-      </c>
-      <c r="C534" t="s">
-        <v>19</v>
-      </c>
-      <c r="D534" t="s">
+      <c r="A534" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B534" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C534" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D534" s="4" t="s">
         <v>498</v>
       </c>
-      <c r="E534">
+      <c r="E534" s="4">
         <v>17628588</v>
       </c>
-      <c r="F534">
+      <c r="F534" s="4">
         <v>95367</v>
       </c>
-      <c r="G534">
+      <c r="G534" s="4">
         <v>72244.429000000004</v>
       </c>
-      <c r="H534">
+      <c r="H534" s="4">
         <v>493693</v>
       </c>
-      <c r="I534">
+      <c r="I534" s="4">
         <v>2997</v>
       </c>
-      <c r="J534">
+      <c r="J534" s="4">
         <v>2025.4290000000001</v>
       </c>
-      <c r="K534">
+      <c r="K534" s="4">
         <v>81874.047000000006</v>
       </c>
-      <c r="L534">
+      <c r="L534" s="4">
         <v>442.92200000000003</v>
       </c>
-      <c r="M534">
+      <c r="M534" s="4">
         <v>335.53100000000001</v>
       </c>
-      <c r="N534">
+      <c r="N534" s="4">
         <v>2292.9029999999998</v>
       </c>
-      <c r="O534">
+      <c r="O534" s="4">
         <v>13.919</v>
       </c>
-      <c r="P534">
+      <c r="P534" s="4">
         <v>9.407</v>
       </c>
-      <c r="Q534">
+      <c r="Q534" s="4">
         <v>1</v>
       </c>
     </row>
     <row r="535" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A535" t="s">
-        <v>17</v>
-      </c>
-      <c r="B535" t="s">
-        <v>18</v>
-      </c>
-      <c r="C535" t="s">
-        <v>19</v>
-      </c>
-      <c r="D535" t="s">
+      <c r="A535" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B535" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C535" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D535" s="4" t="s">
         <v>499</v>
       </c>
-      <c r="E535">
+      <c r="E535" s="4">
         <v>17702630</v>
       </c>
-      <c r="F535">
+      <c r="F535" s="4">
         <v>74042</v>
       </c>
-      <c r="G535">
+      <c r="G535" s="4">
         <v>70237.285999999993</v>
       </c>
-      <c r="H535">
+      <c r="H535" s="4">
         <v>496004</v>
       </c>
-      <c r="I535">
+      <c r="I535" s="4">
         <v>2311</v>
       </c>
-      <c r="J535">
+      <c r="J535" s="4">
         <v>1997.857</v>
       </c>
-      <c r="K535">
+      <c r="K535" s="4">
         <v>82217.926999999996</v>
       </c>
-      <c r="L535">
+      <c r="L535" s="4">
         <v>343.88</v>
       </c>
-      <c r="M535">
+      <c r="M535" s="4">
         <v>326.209</v>
       </c>
-      <c r="N535">
+      <c r="N535" s="4">
         <v>2303.636</v>
       </c>
-      <c r="O535">
+      <c r="O535" s="4">
         <v>10.733000000000001</v>
       </c>
-      <c r="P535">
+      <c r="P535" s="4">
         <v>9.2789999999999999</v>
       </c>
-      <c r="Q535">
+      <c r="Q535" s="4">
         <v>0.99</v>
       </c>
     </row>
     <row r="536" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A536" t="s">
-        <v>17</v>
-      </c>
-      <c r="B536" t="s">
-        <v>18</v>
-      </c>
-      <c r="C536" t="s">
-        <v>19</v>
-      </c>
-      <c r="D536" t="s">
+      <c r="A536" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B536" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C536" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D536" s="4" t="s">
         <v>500</v>
       </c>
-      <c r="E536">
+      <c r="E536" s="4">
         <v>17801462</v>
       </c>
-      <c r="F536">
+      <c r="F536" s="4">
         <v>98832</v>
       </c>
-      <c r="G536">
+      <c r="G536" s="4">
         <v>72192</v>
       </c>
-      <c r="H536">
+      <c r="H536" s="4">
         <v>498499</v>
       </c>
-      <c r="I536">
+      <c r="I536" s="4">
         <v>2495</v>
       </c>
-      <c r="J536">
+      <c r="J536" s="4">
         <v>2037.7139999999999</v>
       </c>
-      <c r="K536">
+      <c r="K536" s="4">
         <v>82676.941999999995</v>
       </c>
-      <c r="L536">
+      <c r="L536" s="4">
         <v>459.01400000000001</v>
       </c>
-      <c r="M536">
+      <c r="M536" s="4">
         <v>335.28800000000001</v>
       </c>
-      <c r="N536">
+      <c r="N536" s="4">
         <v>2315.2240000000002</v>
       </c>
-      <c r="O536">
+      <c r="O536" s="4">
         <v>11.587999999999999</v>
       </c>
-      <c r="P536">
+      <c r="P536" s="4">
         <v>9.4640000000000004</v>
       </c>
-      <c r="Q536">
+      <c r="Q536" s="4">
         <v>0.99</v>
       </c>
     </row>
     <row r="537" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A537" t="s">
-        <v>17</v>
-      </c>
-      <c r="B537" t="s">
-        <v>18</v>
-      </c>
-      <c r="C537" t="s">
-        <v>19</v>
-      </c>
-      <c r="D537" t="s">
+      <c r="A537" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B537" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C537" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D537" s="4" t="s">
         <v>501</v>
       </c>
-      <c r="E537">
+      <c r="E537" s="4">
         <v>17883750</v>
       </c>
-      <c r="F537">
+      <c r="F537" s="4">
         <v>82288</v>
       </c>
-      <c r="G537">
+      <c r="G537" s="4">
         <v>72704.570999999996</v>
       </c>
-      <c r="H537">
+      <c r="H537" s="4">
         <v>500800</v>
       </c>
-      <c r="I537">
+      <c r="I537" s="4">
         <v>2301</v>
       </c>
-      <c r="J537">
+      <c r="J537" s="4">
         <v>2075.4290000000001</v>
       </c>
-      <c r="K537">
+      <c r="K537" s="4">
         <v>83059.119000000006</v>
       </c>
-      <c r="L537">
+      <c r="L537" s="4">
         <v>382.178</v>
       </c>
-      <c r="M537">
+      <c r="M537" s="4">
         <v>337.66800000000001</v>
       </c>
-      <c r="N537">
+      <c r="N537" s="4">
         <v>2325.9110000000001</v>
       </c>
-      <c r="O537">
+      <c r="O537" s="4">
         <v>10.686999999999999</v>
       </c>
-      <c r="P537">
+      <c r="P537" s="4">
         <v>9.6389999999999993</v>
       </c>
-      <c r="Q537">
+      <c r="Q537" s="4">
         <v>0.98</v>
       </c>
     </row>
     <row r="538" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A538" t="s">
-        <v>17</v>
-      </c>
-      <c r="B538" t="s">
-        <v>18</v>
-      </c>
-      <c r="C538" t="s">
-        <v>19</v>
-      </c>
-      <c r="D538" t="s">
+      <c r="A538" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B538" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C538" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D538" s="4" t="s">
         <v>502</v>
       </c>
-      <c r="E538">
+      <c r="E538" s="4">
         <v>17927928</v>
       </c>
-      <c r="F538">
+      <c r="F538" s="4">
         <v>44178</v>
       </c>
-      <c r="G538">
+      <c r="G538" s="4">
         <v>73594.570999999996</v>
       </c>
-      <c r="H538">
+      <c r="H538" s="4">
         <v>501825</v>
       </c>
-      <c r="I538">
+      <c r="I538" s="4">
         <v>1025</v>
       </c>
-      <c r="J538">
+      <c r="J538" s="4">
         <v>2060.5709999999999</v>
       </c>
-      <c r="K538">
+      <c r="K538" s="4">
         <v>83264.298999999999</v>
       </c>
-      <c r="L538">
+      <c r="L538" s="4">
         <v>205.18</v>
       </c>
-      <c r="M538">
+      <c r="M538" s="4">
         <v>341.80200000000002</v>
       </c>
-      <c r="N538">
+      <c r="N538" s="4">
         <v>2330.6709999999998</v>
       </c>
-      <c r="O538">
+      <c r="O538" s="4">
         <v>4.7610000000000001</v>
       </c>
-      <c r="P538">
+      <c r="P538" s="4">
         <v>9.57</v>
       </c>
-      <c r="Q538">
+      <c r="Q538" s="4">
         <v>0.98</v>
       </c>
     </row>
     <row r="539" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A539" t="s">
-        <v>17</v>
-      </c>
-      <c r="B539" t="s">
-        <v>18</v>
-      </c>
-      <c r="C539" t="s">
-        <v>19</v>
-      </c>
-      <c r="D539" t="s">
+      <c r="A539" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B539" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C539" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D539" s="4" t="s">
         <v>503</v>
       </c>
-      <c r="E539">
+      <c r="E539" s="4">
         <v>17966831</v>
       </c>
-      <c r="F539">
+      <c r="F539" s="4">
         <v>38903</v>
       </c>
-      <c r="G539">
+      <c r="G539" s="4">
         <v>73459.857000000004</v>
       </c>
-      <c r="H539">
+      <c r="H539" s="4">
         <v>502586</v>
       </c>
-      <c r="I539">
+      <c r="I539" s="4">
         <v>761</v>
       </c>
-      <c r="J539">
+      <c r="J539" s="4">
         <v>2051.143</v>
       </c>
-      <c r="K539">
+      <c r="K539" s="4">
         <v>83444.98</v>
       </c>
-      <c r="L539">
+      <c r="L539" s="4">
         <v>180.68100000000001</v>
       </c>
-      <c r="M539">
+      <c r="M539" s="4">
         <v>341.17599999999999</v>
       </c>
-      <c r="N539">
+      <c r="N539" s="4">
         <v>2334.2060000000001</v>
       </c>
-      <c r="O539">
+      <c r="O539" s="4">
         <v>3.5339999999999998</v>
       </c>
-      <c r="P539">
+      <c r="P539" s="4">
         <v>9.5259999999999998</v>
       </c>
-      <c r="Q539">
+      <c r="Q539" s="4">
         <v>0.97</v>
       </c>
     </row>
     <row r="540" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A540" t="s">
-        <v>17</v>
-      </c>
-      <c r="B540" t="s">
-        <v>18</v>
-      </c>
-      <c r="C540" t="s">
-        <v>19</v>
-      </c>
-      <c r="D540" t="s">
+      <c r="A540" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B540" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C540" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D540" s="4" t="s">
         <v>504</v>
       </c>
-      <c r="E540">
+      <c r="E540" s="4">
         <v>18054653</v>
       </c>
-      <c r="F540">
+      <c r="F540" s="4">
         <v>87822</v>
       </c>
-      <c r="G540">
+      <c r="G540" s="4">
         <v>74490.285999999993</v>
       </c>
-      <c r="H540">
+      <c r="H540" s="4">
         <v>504717</v>
       </c>
-      <c r="I540">
+      <c r="I540" s="4">
         <v>2131</v>
       </c>
-      <c r="J540">
+      <c r="J540" s="4">
         <v>2003</v>
       </c>
-      <c r="K540">
+      <c r="K540" s="4">
         <v>83852.86</v>
       </c>
-      <c r="L540">
+      <c r="L540" s="4">
         <v>407.88</v>
       </c>
-      <c r="M540">
+      <c r="M540" s="4">
         <v>345.96199999999999</v>
       </c>
-      <c r="N540">
+      <c r="N540" s="4">
         <v>2344.1030000000001</v>
       </c>
-      <c r="O540">
+      <c r="O540" s="4">
         <v>9.8970000000000002</v>
       </c>
-      <c r="P540">
+      <c r="P540" s="4">
         <v>9.3030000000000008</v>
       </c>
-      <c r="Q540">
+      <c r="Q540" s="4">
         <v>0.96</v>
       </c>
     </row>
     <row r="541" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A541" t="s">
-        <v>17</v>
-      </c>
-      <c r="B541" t="s">
-        <v>18</v>
-      </c>
-      <c r="C541" t="s">
-        <v>19</v>
-      </c>
-      <c r="D541" t="s">
+      <c r="A541" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B541" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C541" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D541" s="4" t="s">
         <v>505</v>
       </c>
-      <c r="E541">
+      <c r="E541" s="4">
         <v>18169881</v>
       </c>
-      <c r="F541">
+      <c r="F541" s="4">
         <v>115228</v>
       </c>
-      <c r="G541">
+      <c r="G541" s="4">
         <v>77327.570999999996</v>
       </c>
-      <c r="H541">
+      <c r="H541" s="4">
         <v>507109</v>
       </c>
-      <c r="I541">
+      <c r="I541" s="4">
         <v>2392</v>
       </c>
-      <c r="J541">
+      <c r="J541" s="4">
         <v>1916.5709999999999</v>
       </c>
-      <c r="K541">
+      <c r="K541" s="4">
         <v>84388.023000000001</v>
       </c>
-      <c r="L541">
+      <c r="L541" s="4">
         <v>535.16399999999999</v>
       </c>
-      <c r="M541">
+      <c r="M541" s="4">
         <v>359.13900000000001</v>
       </c>
-      <c r="N541">
+      <c r="N541" s="4">
         <v>2355.212</v>
       </c>
-      <c r="O541">
+      <c r="O541" s="4">
         <v>11.109</v>
       </c>
-      <c r="P541">
+      <c r="P541" s="4">
         <v>8.9009999999999998</v>
       </c>
-      <c r="Q541">
+      <c r="Q541" s="4">
         <v>0.95</v>
       </c>
     </row>
     <row r="542" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A542" t="s">
-        <v>17</v>
-      </c>
-      <c r="B542" t="s">
-        <v>18</v>
-      </c>
-      <c r="C542" t="s">
-        <v>19</v>
-      </c>
-      <c r="D542" t="s">
+      <c r="A542" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B542" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C542" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D542" s="4" t="s">
         <v>506</v>
       </c>
-      <c r="E542">
+      <c r="E542" s="4">
         <v>18243483</v>
       </c>
-      <c r="F542">
+      <c r="F542" s="4">
         <v>73602</v>
       </c>
-      <c r="G542">
+      <c r="G542" s="4">
         <v>77264.714000000007</v>
       </c>
-      <c r="H542">
+      <c r="H542" s="4">
         <v>509141</v>
       </c>
-      <c r="I542">
+      <c r="I542" s="4">
         <v>2032</v>
       </c>
-      <c r="J542">
+      <c r="J542" s="4">
         <v>1876.7139999999999</v>
       </c>
-      <c r="K542">
+      <c r="K542" s="4">
         <v>84729.86</v>
       </c>
-      <c r="L542">
+      <c r="L542" s="4">
         <v>341.83600000000001</v>
       </c>
-      <c r="M542">
+      <c r="M542" s="4">
         <v>358.84800000000001</v>
       </c>
-      <c r="N542">
+      <c r="N542" s="4">
         <v>2364.65</v>
       </c>
-      <c r="O542">
+      <c r="O542" s="4">
         <v>9.4369999999999994</v>
       </c>
-      <c r="P542">
+      <c r="P542" s="4">
         <v>8.7159999999999993</v>
       </c>
-      <c r="Q542">
+      <c r="Q542" s="4">
         <v>0.94</v>
       </c>
     </row>
     <row r="543" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A543" t="s">
-        <v>17</v>
-      </c>
-      <c r="B543" t="s">
-        <v>18</v>
-      </c>
-      <c r="C543" t="s">
-        <v>19</v>
-      </c>
-      <c r="D543" t="s">
+      <c r="A543" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B543" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C543" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D543" s="4" t="s">
         <v>507</v>
       </c>
-      <c r="E543">
+      <c r="E543" s="4">
         <v>18322760</v>
       </c>
-      <c r="F543">
+      <c r="F543" s="4">
         <v>79277</v>
       </c>
-      <c r="G543">
+      <c r="G543" s="4">
         <v>74471.142999999996</v>
       </c>
-      <c r="H543">
+      <c r="H543" s="4">
         <v>511142</v>
       </c>
-      <c r="I543">
+      <c r="I543" s="4">
         <v>2001</v>
       </c>
-      <c r="J543">
+      <c r="J543" s="4">
         <v>1806.143</v>
       </c>
-      <c r="K543">
+      <c r="K543" s="4">
         <v>85098.053</v>
       </c>
-      <c r="L543">
+      <c r="L543" s="4">
         <v>368.19299999999998</v>
       </c>
-      <c r="M543">
+      <c r="M543" s="4">
         <v>345.87299999999999</v>
       </c>
-      <c r="N543">
+      <c r="N543" s="4">
         <v>2373.9430000000002</v>
       </c>
-      <c r="O543">
+      <c r="O543" s="4">
         <v>9.2929999999999993</v>
       </c>
-      <c r="P543">
+      <c r="P543" s="4">
         <v>8.3879999999999999</v>
       </c>
-      <c r="Q543">
+      <c r="Q543" s="4">
         <v>0.94</v>
       </c>
     </row>
     <row r="544" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A544" t="s">
-        <v>17</v>
-      </c>
-      <c r="B544" t="s">
-        <v>18</v>
-      </c>
-      <c r="C544" t="s">
-        <v>19</v>
-      </c>
-      <c r="D544" t="s">
+      <c r="A544" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B544" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C544" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D544" s="4" t="s">
         <v>508</v>
       </c>
-      <c r="E544">
+      <c r="E544" s="4">
         <v>18386894</v>
       </c>
-      <c r="F544">
+      <c r="F544" s="4">
         <v>64134</v>
       </c>
-      <c r="G544">
+      <c r="G544" s="4">
         <v>71877.714000000007</v>
       </c>
-      <c r="H544">
+      <c r="H544" s="4">
         <v>512735</v>
       </c>
-      <c r="I544">
+      <c r="I544" s="4">
         <v>1593</v>
       </c>
-      <c r="J544">
+      <c r="J544" s="4">
         <v>1705</v>
       </c>
-      <c r="K544">
+      <c r="K544" s="4">
         <v>85395.915999999997</v>
       </c>
-      <c r="L544">
+      <c r="L544" s="4">
         <v>297.863</v>
       </c>
-      <c r="M544">
+      <c r="M544" s="4">
         <v>333.82799999999997</v>
       </c>
-      <c r="N544">
+      <c r="N544" s="4">
         <v>2381.3420000000001</v>
       </c>
-      <c r="O544">
+      <c r="O544" s="4">
         <v>7.399</v>
       </c>
-      <c r="P544">
+      <c r="P544" s="4">
         <v>7.9189999999999996</v>
       </c>
-      <c r="Q544">
+      <c r="Q544" s="4">
         <v>0.93</v>
       </c>
     </row>
     <row r="545" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A545" t="s">
-        <v>17</v>
-      </c>
-      <c r="B545" t="s">
-        <v>18</v>
-      </c>
-      <c r="C545" t="s">
-        <v>19</v>
-      </c>
-      <c r="D545" t="s">
+      <c r="A545" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B545" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C545" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D545" s="4" t="s">
         <v>509</v>
       </c>
-      <c r="E545">
+      <c r="E545" s="4">
         <v>18420598</v>
       </c>
-      <c r="F545">
+      <c r="F545" s="4">
         <v>33704</v>
       </c>
-      <c r="G545">
+      <c r="G545" s="4">
         <v>70381.429000000004</v>
       </c>
-      <c r="H545">
+      <c r="H545" s="4">
         <v>513474</v>
       </c>
-      <c r="I545">
+      <c r="I545" s="4">
         <v>739</v>
       </c>
-      <c r="J545">
+      <c r="J545" s="4">
         <v>1664.143</v>
       </c>
-      <c r="K545">
+      <c r="K545" s="4">
         <v>85552.451000000001</v>
       </c>
-      <c r="L545">
+      <c r="L545" s="4">
         <v>156.535</v>
       </c>
-      <c r="M545">
+      <c r="M545" s="4">
         <v>326.87900000000002</v>
       </c>
-      <c r="N545">
+      <c r="N545" s="4">
         <v>2384.7739999999999</v>
       </c>
-      <c r="O545">
+      <c r="O545" s="4">
         <v>3.4319999999999999</v>
       </c>
-      <c r="P545">
+      <c r="P545" s="4">
         <v>7.7290000000000001</v>
       </c>
-      <c r="Q545">
+      <c r="Q545" s="4">
         <v>0.92</v>
       </c>
     </row>
     <row r="546" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A546" t="s">
-        <v>17</v>
-      </c>
-      <c r="B546" t="s">
-        <v>18</v>
-      </c>
-      <c r="C546" t="s">
-        <v>19</v>
-      </c>
-      <c r="D546" t="s">
+      <c r="A546" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B546" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C546" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D546" s="4" t="s">
         <v>510</v>
       </c>
-      <c r="E546">
+      <c r="E546" s="4">
         <v>18448402</v>
       </c>
-      <c r="F546">
+      <c r="F546" s="4">
         <v>27804</v>
       </c>
-      <c r="G546">
+      <c r="G546" s="4">
         <v>68795.857000000004</v>
       </c>
-      <c r="H546">
+      <c r="H546" s="4">
         <v>514092</v>
       </c>
-      <c r="I546">
+      <c r="I546" s="4">
         <v>618</v>
       </c>
-      <c r="J546">
+      <c r="J546" s="4">
         <v>1643.7139999999999</v>
       </c>
-      <c r="K546">
+      <c r="K546" s="4">
         <v>85681.584000000003</v>
       </c>
-      <c r="L546">
+      <c r="L546" s="4">
         <v>129.13300000000001</v>
       </c>
-      <c r="M546">
+      <c r="M546" s="4">
         <v>319.51499999999999</v>
       </c>
-      <c r="N546">
+      <c r="N546" s="4">
         <v>2387.6439999999998</v>
       </c>
-      <c r="O546">
+      <c r="O546" s="4">
         <v>2.87</v>
       </c>
-      <c r="P546">
+      <c r="P546" s="4">
         <v>7.6340000000000003</v>
       </c>
-      <c r="Q546">
+      <c r="Q546" s="4">
         <v>0.92</v>
       </c>
     </row>
     <row r="547" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A547" t="s">
-        <v>17</v>
-      </c>
-      <c r="B547" t="s">
-        <v>18</v>
-      </c>
-      <c r="C547" t="s">
-        <v>19</v>
-      </c>
-      <c r="D547" t="s">
+      <c r="A547" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B547" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C547" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D547" s="6" t="s">
         <v>511</v>
       </c>
-      <c r="E547">
+      <c r="E547" s="6">
         <v>18513305</v>
       </c>
-      <c r="F547">
+      <c r="F547" s="6">
         <v>64903</v>
       </c>
-      <c r="G547">
+      <c r="G547" s="6">
         <v>65521.714</v>
       </c>
-      <c r="H547">
+      <c r="H547" s="6">
         <v>515985</v>
       </c>
-      <c r="I547">
+      <c r="I547" s="6">
         <v>1893</v>
       </c>
-      <c r="J547">
+      <c r="J547" s="6">
         <v>1609.7139999999999</v>
       </c>
-      <c r="K547">
+      <c r="K547" s="6">
         <v>85983.019</v>
       </c>
-      <c r="L547">
+      <c r="L547" s="6">
         <v>301.435</v>
       </c>
-      <c r="M547">
+      <c r="M547" s="6">
         <v>304.30799999999999</v>
       </c>
-      <c r="N547">
+      <c r="N547" s="6">
         <v>2396.4360000000001</v>
       </c>
-      <c r="O547">
+      <c r="O547" s="6">
         <v>8.7919999999999998</v>
       </c>
-      <c r="P547">
+      <c r="P547" s="6">
         <v>7.476</v>
       </c>
-      <c r="Q547">
+      <c r="Q547" s="6">
         <v>0.92</v>
       </c>
     </row>
     <row r="548" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A548" t="s">
-        <v>17</v>
-      </c>
-      <c r="B548" t="s">
-        <v>18</v>
-      </c>
-      <c r="C548" t="s">
-        <v>19</v>
-      </c>
-      <c r="D548" t="s">
+      <c r="A548" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B548" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C548" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D548" s="6" t="s">
         <v>512</v>
       </c>
-      <c r="E548">
+      <c r="E548" s="6">
         <v>18557141</v>
       </c>
-      <c r="F548">
+      <c r="F548" s="6">
         <v>43836</v>
       </c>
-      <c r="G548">
+      <c r="G548" s="6">
         <v>55322.857000000004</v>
       </c>
-      <c r="H548">
+      <c r="H548" s="6">
         <v>518066</v>
       </c>
-      <c r="I548">
+      <c r="I548" s="6">
         <v>2081</v>
       </c>
-      <c r="J548">
+      <c r="J548" s="6">
         <v>1565.2860000000001</v>
       </c>
-      <c r="K548">
+      <c r="K548" s="6">
         <v>86186.61</v>
       </c>
-      <c r="L548">
+      <c r="L548" s="6">
         <v>203.59200000000001</v>
       </c>
-      <c r="M548">
+      <c r="M548" s="6">
         <v>256.94099999999997</v>
       </c>
-      <c r="N548">
+      <c r="N548" s="6">
         <v>2406.1010000000001</v>
       </c>
-      <c r="O548">
+      <c r="O548" s="6">
         <v>9.6649999999999991</v>
       </c>
-      <c r="P548">
+      <c r="P548" s="6">
         <v>7.27</v>
       </c>
-      <c r="Q548">
+      <c r="Q548" s="6">
         <v>0.92</v>
       </c>
     </row>
     <row r="549" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A549" t="s">
-        <v>17</v>
-      </c>
-      <c r="B549" t="s">
-        <v>18</v>
-      </c>
-      <c r="C549" t="s">
-        <v>19</v>
-      </c>
-      <c r="D549" t="s">
+      <c r="A549" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B549" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C549" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D549" s="6" t="s">
         <v>513</v>
       </c>
-      <c r="E549">
+      <c r="E549" s="6">
         <v>18622304</v>
       </c>
-      <c r="F549">
+      <c r="F549" s="6">
         <v>65163</v>
       </c>
-      <c r="G549">
+      <c r="G549" s="6">
         <v>54117.286</v>
       </c>
-      <c r="H549">
+      <c r="H549" s="6">
         <v>520095</v>
       </c>
-      <c r="I549">
+      <c r="I549" s="6">
         <v>2029</v>
       </c>
-      <c r="J549">
+      <c r="J549" s="6">
         <v>1564.857</v>
       </c>
-      <c r="K549">
+      <c r="K549" s="6">
         <v>86489.251999999993</v>
       </c>
-      <c r="L549">
+      <c r="L549" s="6">
         <v>302.642</v>
       </c>
-      <c r="M549">
+      <c r="M549" s="6">
         <v>251.34200000000001</v>
       </c>
-      <c r="N549">
+      <c r="N549" s="6">
         <v>2415.5239999999999</v>
       </c>
-      <c r="O549">
+      <c r="O549" s="6">
         <v>9.423</v>
       </c>
-      <c r="P549">
+      <c r="P549" s="6">
         <v>7.2679999999999998</v>
       </c>
-      <c r="Q549">
+      <c r="Q549" s="6">
         <v>0.92</v>
       </c>
     </row>
     <row r="550" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A550" t="s">
-        <v>17</v>
-      </c>
-      <c r="B550" t="s">
-        <v>18</v>
-      </c>
-      <c r="C550" t="s">
-        <v>19</v>
-      </c>
-      <c r="D550" t="s">
+      <c r="A550" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B550" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C550" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D550" s="6" t="s">
         <v>514</v>
       </c>
-      <c r="E550">
+      <c r="E550" s="6">
         <v>18687469</v>
       </c>
-      <c r="F550">
+      <c r="F550" s="6">
         <v>65165</v>
       </c>
-      <c r="G550">
+      <c r="G550" s="6">
         <v>52101.286</v>
       </c>
-      <c r="H550">
+      <c r="H550" s="6">
         <v>521952</v>
       </c>
-      <c r="I550">
+      <c r="I550" s="6">
         <v>1857</v>
       </c>
-      <c r="J550">
+      <c r="J550" s="6">
         <v>1544.2860000000001</v>
       </c>
-      <c r="K550">
+      <c r="K550" s="6">
         <v>86791.903999999995</v>
       </c>
-      <c r="L550">
+      <c r="L550" s="6">
         <v>302.65199999999999</v>
       </c>
-      <c r="M550">
+      <c r="M550" s="6">
         <v>241.97900000000001</v>
       </c>
-      <c r="N550">
+      <c r="N550" s="6">
         <v>2424.1489999999999</v>
       </c>
-      <c r="O550">
+      <c r="O550" s="6">
         <v>8.625</v>
       </c>
-      <c r="P550">
+      <c r="P550" s="6">
         <v>7.1719999999999997</v>
       </c>
-      <c r="Q550">
+      <c r="Q550" s="6">
         <v>0.91</v>
       </c>
     </row>
     <row r="551" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A551" t="s">
-        <v>17</v>
-      </c>
-      <c r="B551" t="s">
-        <v>18</v>
-      </c>
-      <c r="C551" t="s">
-        <v>19</v>
-      </c>
-      <c r="D551" t="s">
+      <c r="A551" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B551" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C551" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D551" s="6" t="s">
         <v>515</v>
       </c>
-      <c r="E551">
+      <c r="E551" s="6">
         <v>18742025</v>
       </c>
-      <c r="F551">
+      <c r="F551" s="6">
         <v>54556</v>
       </c>
-      <c r="G551">
+      <c r="G551" s="6">
         <v>50733</v>
       </c>
-      <c r="H551">
+      <c r="H551" s="6">
         <v>523587</v>
       </c>
-      <c r="I551">
+      <c r="I551" s="6">
         <v>1635</v>
       </c>
-      <c r="J551">
+      <c r="J551" s="6">
         <v>1550.2860000000001</v>
       </c>
-      <c r="K551">
+      <c r="K551" s="6">
         <v>87045.284</v>
       </c>
-      <c r="L551">
+      <c r="L551" s="6">
         <v>253.37899999999999</v>
       </c>
-      <c r="M551">
+      <c r="M551" s="6">
         <v>235.624</v>
       </c>
-      <c r="N551">
+      <c r="N551" s="6">
         <v>2431.7429999999999</v>
       </c>
-      <c r="O551">
+      <c r="O551" s="6">
         <v>7.5940000000000003</v>
       </c>
-      <c r="P551">
+      <c r="P551" s="6">
         <v>7.2</v>
       </c>
-      <c r="Q551">
+      <c r="Q551" s="6">
         <v>0.91</v>
       </c>
     </row>
     <row r="552" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A552" t="s">
-        <v>17</v>
-      </c>
-      <c r="B552" t="s">
-        <v>18</v>
-      </c>
-      <c r="C552" t="s">
-        <v>19</v>
-      </c>
-      <c r="D552" t="s">
+      <c r="A552" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B552" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C552" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D552" s="6" t="s">
         <v>516</v>
       </c>
-      <c r="E552">
+      <c r="E552" s="6">
         <v>18769808</v>
       </c>
-      <c r="F552">
+      <c r="F552" s="6">
         <v>27783</v>
       </c>
-      <c r="G552">
+      <c r="G552" s="6">
         <v>49887.142999999996</v>
       </c>
-      <c r="H552">
+      <c r="H552" s="6">
         <v>524417</v>
       </c>
-      <c r="I552">
+      <c r="I552" s="6">
         <v>830</v>
       </c>
-      <c r="J552">
+      <c r="J552" s="6">
         <v>1563.2860000000001</v>
       </c>
-      <c r="K552">
+      <c r="K552" s="6">
         <v>87174.319000000003</v>
       </c>
-      <c r="L552">
+      <c r="L552" s="6">
         <v>129.035</v>
       </c>
-      <c r="M552">
+      <c r="M552" s="6">
         <v>231.69499999999999</v>
       </c>
-      <c r="N552">
+      <c r="N552" s="6">
         <v>2435.5970000000002</v>
       </c>
-      <c r="O552">
+      <c r="O552" s="6">
         <v>3.855</v>
       </c>
-      <c r="P552">
+      <c r="P552" s="6">
         <v>7.2610000000000001</v>
       </c>
-      <c r="Q552">
+      <c r="Q552" s="6">
         <v>0.91</v>
       </c>
     </row>
     <row r="553" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A553" t="s">
-        <v>17</v>
-      </c>
-      <c r="B553" t="s">
-        <v>18</v>
-      </c>
-      <c r="C553" t="s">
-        <v>19</v>
-      </c>
-      <c r="D553" t="s">
+      <c r="A553" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B553" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C553" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D553" s="6" t="s">
         <v>517</v>
       </c>
-      <c r="E553">
+      <c r="E553" s="6">
         <v>18792511</v>
       </c>
-      <c r="F553">
+      <c r="F553" s="6">
         <v>22703</v>
       </c>
-      <c r="G553">
+      <c r="G553" s="6">
         <v>49158.428999999996</v>
       </c>
-      <c r="H553">
+      <c r="H553" s="6">
         <v>525112</v>
       </c>
-      <c r="I553">
+      <c r="I553" s="6">
         <v>695</v>
       </c>
-      <c r="J553">
+      <c r="J553" s="6">
         <v>1574.2860000000001</v>
       </c>
-      <c r="K553">
+      <c r="K553" s="6">
         <v>87279.76</v>
       </c>
-      <c r="L553">
+      <c r="L553" s="6">
         <v>105.44199999999999</v>
       </c>
-      <c r="M553">
+      <c r="M553" s="6">
         <v>228.31100000000001</v>
       </c>
-      <c r="N553">
+      <c r="N553" s="6">
         <v>2438.8249999999998</v>
       </c>
-      <c r="O553">
+      <c r="O553" s="6">
         <v>3.2280000000000002</v>
       </c>
-      <c r="P553">
+      <c r="P553" s="6">
         <v>7.3120000000000003</v>
       </c>
-      <c r="Q553">
+      <c r="Q553" s="6">
         <v>0.91</v>
       </c>
     </row>
     <row r="554" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A554" t="s">
-        <v>17</v>
-      </c>
-      <c r="B554" t="s">
-        <v>18</v>
-      </c>
-      <c r="C554" t="s">
-        <v>19</v>
-      </c>
-      <c r="D554" t="s">
+      <c r="A554" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B554" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C554" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D554" s="6" t="s">
         <v>518</v>
       </c>
-      <c r="E554">
+      <c r="E554" s="6">
         <v>18855015</v>
       </c>
-      <c r="F554">
+      <c r="F554" s="6">
         <v>62504</v>
       </c>
-      <c r="G554">
+      <c r="G554" s="6">
         <v>48815.714</v>
       </c>
-      <c r="H554">
+      <c r="H554" s="6">
         <v>526892</v>
       </c>
-      <c r="I554">
+      <c r="I554" s="6">
         <v>1780</v>
       </c>
-      <c r="J554">
+      <c r="J554" s="6">
         <v>1558.143</v>
       </c>
-      <c r="K554">
+      <c r="K554" s="6">
         <v>87570.053</v>
       </c>
-      <c r="L554">
+      <c r="L554" s="6">
         <v>290.29300000000001</v>
       </c>
-      <c r="M554">
+      <c r="M554" s="6">
         <v>226.71899999999999</v>
       </c>
-      <c r="N554">
+      <c r="N554" s="6">
         <v>2447.0920000000001</v>
       </c>
-      <c r="O554">
+      <c r="O554" s="6">
         <v>8.2669999999999995</v>
       </c>
-      <c r="P554">
+      <c r="P554" s="6">
         <v>7.2370000000000001</v>
       </c>
-      <c r="Q554">
+      <c r="Q554" s="6">
         <v>0.91</v>
       </c>
     </row>
     <row r="555" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A555" t="s">
-        <v>17</v>
-      </c>
-      <c r="B555" t="s">
-        <v>18</v>
-      </c>
-      <c r="C555" t="s">
-        <v>19</v>
-      </c>
-      <c r="D555" t="s">
+      <c r="A555" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B555" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C555" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D555" s="6" t="s">
         <v>519</v>
       </c>
-      <c r="E555">
+      <c r="E555" s="6">
         <v>18909037</v>
       </c>
-      <c r="F555">
+      <c r="F555" s="6">
         <v>54022</v>
       </c>
-      <c r="G555">
+      <c r="G555" s="6">
         <v>50270.857000000004</v>
       </c>
-      <c r="H555">
+      <c r="H555" s="6">
         <v>528540</v>
       </c>
-      <c r="I555">
+      <c r="I555" s="6">
         <v>1648</v>
       </c>
-      <c r="J555">
+      <c r="J555" s="6">
         <v>1496.2860000000001</v>
       </c>
-      <c r="K555">
+      <c r="K555" s="6">
         <v>87820.952000000005</v>
       </c>
-      <c r="L555">
+      <c r="L555" s="6">
         <v>250.899</v>
       </c>
-      <c r="M555">
+      <c r="M555" s="6">
         <v>233.477</v>
       </c>
-      <c r="N555">
+      <c r="N555" s="6">
         <v>2454.7460000000001</v>
       </c>
-      <c r="O555">
+      <c r="O555" s="6">
         <v>7.6539999999999999</v>
       </c>
-      <c r="P555">
+      <c r="P555" s="6">
         <v>6.9489999999999998</v>
       </c>
-      <c r="Q555">
+      <c r="Q555" s="6">
         <v>0.91</v>
       </c>
     </row>
     <row r="556" spans="1:17" x14ac:dyDescent="0.2">
-      <c r="A556" t="s">
-        <v>17</v>
-      </c>
-      <c r="B556" t="s">
-        <v>18</v>
-      </c>
-      <c r="C556" t="s">
-        <v>19</v>
-      </c>
-      <c r="D556" t="s">
+      <c r="A556" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B556" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C556" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="D556" s="6" t="s">
         <v>520</v>
       </c>
-      <c r="E556">
+      <c r="E556" s="6">
         <v>18962762</v>
       </c>
-      <c r="F556">
+      <c r="F556" s="6">
         <v>53725</v>
       </c>
-      <c r="G556">
+      <c r="G556" s="6">
         <v>48636.857000000004</v>
       </c>
-      <c r="H556">
+      <c r="H556" s="6">
         <v>530179</v>
       </c>
-      <c r="I556">
+      <c r="I556" s="6">
         <v>1639</v>
       </c>
-      <c r="J556">
+      <c r="J556" s="6">
         <v>1440.5709999999999</v>
       </c>
-      <c r="K556">
+      <c r="K556" s="6">
         <v>88070.471999999994</v>
       </c>
-      <c r="L556">
+      <c r="L556" s="6">
         <v>249.52</v>
       </c>
-      <c r="M556">
+      <c r="M556" s="6">
         <v>225.88900000000001</v>
       </c>
-      <c r="N556">
+      <c r="N556" s="6">
         <v>2462.3580000000002</v>
       </c>
-      <c r="O556">
+      <c r="O556" s="6">
         <v>7.6120000000000001</v>
       </c>
-      <c r="P556">
+      <c r="P556" s="6">
         <v>6.6909999999999998</v>
       </c>
-      <c r="Q556">
+      <c r="Q556" s="6">
         <v>0.91</v>
       </c>
     </row>

</xml_diff>